<commit_message>
Storage fixes: separate power and energy params, add lifetime to storage_connection, update storage assumptions
</commit_message>
<xml_diff>
--- a/europe/_power/assumptions.xlsx
+++ b/europe/_power/assumptions.xlsx
@@ -1,23 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\31612\MopoProjects\Mopo_WP2_T5_datapipeline_power_20250522\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944A4D63-F1A1-4425-94B0-10A71B021E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="technology" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="storage" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="technology" sheetId="1" r:id="rId1"/>
+    <sheet name="storage" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
   <si>
     <t>technology</t>
   </si>
@@ -25,16 +29,16 @@
     <t>conversion_rate</t>
   </si>
   <si>
-    <t xml:space="preserve">investment_cost [EUR2020/MWh]</t>
+    <t>investment_cost [EUR2020/MWh]</t>
   </si>
   <si>
     <t>lifetime</t>
   </si>
   <si>
-    <t xml:space="preserve">fixed_cost [% investment]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">operational_cost [EUR2020/MWh]</t>
+    <t>fixed_cost [% investment]</t>
+  </si>
+  <si>
+    <t>operational_cost [EUR2020/MWh]</t>
   </si>
   <si>
     <t>CO2_captured</t>
@@ -73,7 +77,7 @@
     <t>https://www.sciencedirect.com/science/article/pii/S0360319924023681</t>
   </si>
   <si>
-    <t xml:space="preserve">H2-fired OCGT: started from DEA natural-gas OCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024) for H2 GT plants. Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
+    <t>H2-fired OCGT: started from DEA natural-gas OCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024) for H2 GT plants. Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
   </si>
   <si>
     <t>OCGT+CC</t>
@@ -91,7 +95,7 @@
     <t>CCGT-H2</t>
   </si>
   <si>
-    <t xml:space="preserve">H2-fired CCGT: started from DEA natural-gas CCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024). Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
+    <t>H2-fired CCGT: started from DEA natural-gas CCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024). Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
   </si>
   <si>
     <t>CCGT+CC</t>
@@ -103,19 +107,19 @@
     <t>https://ens.dk/sites/ens.dk/files/Statistik/technology_data_for_el_and_dh_13.xlsx</t>
   </si>
   <si>
-    <t xml:space="preserve">Base SCPC O&amp;M + efficiency from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
+    <t>Base SCPC O&amp;M + efficiency from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
   </si>
   <si>
     <t>bioST</t>
   </si>
   <si>
-    <t xml:space="preserve">Bio steam turbine proxied by DEA 'Biomass CHP - extraction - wood chips - large' (May 2025 Excel).</t>
+    <t>Bio steam turbine proxied by DEA 'Biomass CHP - extraction - wood chips - large' (May 2025 Excel).</t>
   </si>
   <si>
     <t>fuelcell</t>
   </si>
   <si>
-    <t xml:space="preserve">Hydrogen fuel cell proxied by DEA 'Low temp PEM fuel cell - back pressure - hydrogen - small' (May 2025 Excel). Variable O&amp;M = 0 in DEA.</t>
+    <t>Hydrogen fuel cell proxied by DEA 'Low temp PEM fuel cell - back pressure - hydrogen - small' (May 2025 Excel). Variable O&amp;M = 0 in DEA.</t>
   </si>
   <si>
     <t>geothermal</t>
@@ -127,7 +131,7 @@
     <t>https://www.irs.gov/individuals/international-taxpayers/yearly-average-currency-exchange-rates</t>
   </si>
   <si>
-    <t xml:space="preserve">Geothermal fixed O&amp;M from NREL ATB 2024 Geothermal (Hydro/Flash). Converted from 2022 $/kW-yr to EUR/MW-yr using IRS 2022 yearly average (1 USD = 0.951 EUR). Variable O&amp;M assumed 0 (not provided in ATB summary). | Conversion rate set to 12% as representative average across DEA geothermal electricity datasheets (2–5 km depth). DEA reports net electrical efficiencies roughly 10–15% depending on depth; midpoint used. | CAPEX from DEA geothermal electricity datasheets (2–5 km depth). Reported range ≈3–6 M€/MW depending on depth and drilling cost; 4.5 M€/MW used as representative average.</t>
+    <t>Geothermal fixed O&amp;M from NREL ATB 2024 Geothermal (Hydro/Flash). Converted from 2022 $/kW-yr to EUR/MW-yr using IRS 2022 yearly average (1 USD = 0.951 EUR). Variable O&amp;M assumed 0 (not provided in ATB summary). | Conversion rate set to 12% as representative average across DEA geothermal electricity datasheets (2–5 km depth). DEA reports net electrical efficiencies roughly 10–15% depending on depth; midpoint used. | CAPEX from DEA geothermal electricity datasheets (2–5 km depth). Reported range ≈3–6 M€/MW depending on depth and drilling cost; 4.5 M€/MW used as representative average.</t>
   </si>
   <si>
     <t>wasteST</t>
@@ -139,10 +143,7 @@
     <t>efficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">investment_cost [EUR/MWh]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">operational_cost [EUR/MWh]</t>
+    <t>operational_cost [EUR/MWh]</t>
   </si>
   <si>
     <t>battery-storage</t>
@@ -154,36 +155,61 @@
     <t>https://ens.dk/media/6589/download</t>
   </si>
   <si>
-    <t xml:space="preserve">DEA Energy Storage datasheet '180 Lithium Ion Battery' (Utility-scale). Efficiencies from charge/discharge; capex from 'Specific investment [MEUR2020/MWh]' (2025 ctrl).</t>
+    <t>DEA Energy Storage datasheet '180 Lithium Ion Battery' (Utility-scale). Efficiencies from charge/discharge; capex from 'Specific investment [MEUR2020/MWh]' (2025 ctrl).</t>
   </si>
   <si>
     <t>battery-storage-iron-air</t>
   </si>
   <si>
-    <t>https://nmreta.com/wp-content/uploads/2022/10/Molly-Bales-Form-Energy-Iron-Air-Battery-Technology.pdf</t>
-  </si>
-  <si>
     <t>https://www.pv-magazine.com/2023/07/14/former-us-coal-plant-to-host-100-hour-iron-air-battery/</t>
   </si>
   <si>
-    <t xml:space="preserve">Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). | Set eff_in=eff_out=sqrt(RTE) assuming symmetric charge/discharge efficiencies. Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
+    <t>Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). | Set eff_in=eff_out=sqrt(RTE) assuming symmetric charge/discharge efficiencies. Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
+  </si>
+  <si>
+    <t>investment_cost_energy [EUR/MWh]</t>
+  </si>
+  <si>
+    <t>investment_cost_power [EUR/MW]</t>
+  </si>
+  <si>
+    <t>fixed_cost_energy [% investment]</t>
+  </si>
+  <si>
+    <t>fixed_cost_power [% investment]</t>
+  </si>
+  <si>
+    <t>https://formenergy.com/technology/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11.000000"/>
+      <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -196,19 +222,23 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -226,291 +256,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -652,70 +399,78 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="19.28515625"/>
-    <col customWidth="1" min="2" max="19" width="18"/>
+    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" customWidth="1"/>
+    <col min="12" max="12" width="16.42578125" customWidth="1"/>
+    <col min="13" max="19" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2">
-        <v>0.40000000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="C2">
         <v>680718.04542770004</v>
@@ -724,7 +479,7 @@
         <v>25</v>
       </c>
       <c r="E2">
-        <v>0.030461610560024992</v>
+        <v>3.0461610560024992E-2</v>
       </c>
       <c r="F2">
         <v>4.6788399592000012</v>
@@ -739,12 +494,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
       <c r="B3">
-        <v>0.40000000000000002</v>
+        <v>0.4</v>
       </c>
       <c r="C3">
         <v>627389.90362</v>
@@ -753,19 +508,19 @@
         <v>25</v>
       </c>
       <c r="E3">
-        <v>0.033050847457627118</v>
+        <v>3.3050847457627118E-2</v>
       </c>
       <c r="F3">
         <v>4.6788399592000012</v>
       </c>
       <c r="G3">
-        <v>0.90000000000000002</v>
+        <v>0.9</v>
       </c>
       <c r="H3">
         <v>0.83299999999999996</v>
       </c>
       <c r="I3">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="J3">
         <v>8.3000000000000007</v>
@@ -786,7 +541,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -800,7 +555,7 @@
         <v>25</v>
       </c>
       <c r="E4">
-        <v>0.030687054880603266</v>
+        <v>3.0687054880603266E-2</v>
       </c>
       <c r="F4">
         <v>4.6788399592000012</v>
@@ -815,7 +570,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -829,19 +584,19 @@
         <v>25</v>
       </c>
       <c r="E5">
-        <v>0.033295454545454538</v>
+        <v>3.3295454545454538E-2</v>
       </c>
       <c r="F5">
         <v>4.6788399592000012</v>
       </c>
       <c r="G5">
-        <v>0.90000000000000002</v>
+        <v>0.9</v>
       </c>
       <c r="H5">
         <v>0.83299999999999996</v>
       </c>
       <c r="I5">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="J5">
         <v>8.3000000000000007</v>
@@ -862,7 +617,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -876,19 +631,19 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>0.0092246335944705105</v>
+        <v>9.2246335944705105E-3</v>
       </c>
       <c r="F6">
         <v>3.279208458421452</v>
       </c>
       <c r="G6">
-        <v>0.90000000000000002</v>
+        <v>0.9</v>
       </c>
       <c r="H6">
         <v>0.83299999999999996</v>
       </c>
       <c r="I6">
-        <v>0.029999999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="J6">
         <v>8.3000000000000007</v>
@@ -909,15 +664,15 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
       <c r="B7">
-        <v>0.42999999999999999</v>
+        <v>0.43</v>
       </c>
       <c r="E7">
-        <v>0.093528001965583196</v>
+        <v>9.3528001965583196E-2</v>
       </c>
       <c r="F7">
         <v>2.7647690668</v>
@@ -929,7 +684,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>31</v>
       </c>
@@ -937,7 +692,7 @@
         <v>0.5</v>
       </c>
       <c r="E8">
-        <v>0.07230044630753138</v>
+        <v>7.230044630753138E-2</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -949,7 +704,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -960,7 +715,7 @@
         <v>4500000</v>
       </c>
       <c r="E9">
-        <v>0.025595773924911289</v>
+        <v>2.5595773924911289E-2</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -975,7 +730,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -984,22 +739,24 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="14.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="22.42578125"/>
-    <col customWidth="1" min="2" max="13" width="18"/>
+    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.5703125" customWidth="1"/>
+    <col min="6" max="15" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
@@ -1009,63 +766,75 @@
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="B2">
+        <v>0.97</v>
+      </c>
+      <c r="C2">
+        <v>0.91</v>
+      </c>
+      <c r="D2">
+        <v>245000</v>
+      </c>
+      <c r="E2">
+        <v>86000</v>
+      </c>
+      <c r="F2">
+        <v>20</v>
+      </c>
+      <c r="G2">
+        <v>3.4299999999999997E-2</v>
+      </c>
+      <c r="H2">
+        <v>9.7699999999999995E-2</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
         <v>42</v>
       </c>
-      <c r="B2">
-        <v>0.96999999999999997</v>
-      </c>
-      <c r="C2">
-        <v>0.91000000000000003</v>
-      </c>
-      <c r="D2">
-        <v>288000</v>
-      </c>
-      <c r="E2">
-        <v>20</v>
-      </c>
-      <c r="F2">
-        <v>0.029000000000000001</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="K2" t="s">
         <v>43</v>
       </c>
-      <c r="I2" t="s">
+      <c r="L2" t="s">
         <v>44</v>
       </c>
-      <c r="J2" t="s">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>46</v>
       </c>
       <c r="B3">
         <v>0.61599999999999999</v>
@@ -1077,25 +846,36 @@
         <v>20000</v>
       </c>
       <c r="E3">
+        <v>550000</v>
+      </c>
+      <c r="F3">
         <v>20</v>
       </c>
-      <c r="F3">
-        <v>0.87780000000000002</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="G3">
+        <v>1E-4</v>
+      </c>
+      <c r="H3">
+        <v>2.9100000000000001E-2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
+        <v>52</v>
+      </c>
+      <c r="K3" t="s">
+        <v>46</v>
+      </c>
+      <c r="L3" t="s">
         <v>47</v>
       </c>
-      <c r="I3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J3" t="s">
-        <v>49</v>
-      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update assumptions file, allow assumptions to overwrite values in jaif
</commit_message>
<xml_diff>
--- a/europe/_power/assumptions.xlsx
+++ b/europe/_power/assumptions.xlsx
@@ -8,15 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\31612\MopoProjects\Mopo_WP2_T5_datapipeline_power_20250522\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{944A4D63-F1A1-4425-94B0-10A71B021E78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920418D8-B034-4064-888A-FD0850D17D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="technology" sheetId="1" r:id="rId1"/>
     <sheet name="storage" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -41,9 +54,6 @@
     <t>operational_cost [EUR2020/MWh]</t>
   </si>
   <si>
-    <t>CO2_captured</t>
-  </si>
-  <si>
     <t>ccs_heat_MWh_per_tCO2</t>
   </si>
   <si>
@@ -180,17 +190,27 @@
   </si>
   <si>
     <t>https://formenergy.com/technology/</t>
+  </si>
+  <si>
+    <t>CO2_captured [tCO2/MWh]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -229,19 +249,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{2E9EB5C5-2F4E-4BFA-85F0-0B749869C9DB}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -438,36 +461,36 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2">
         <v>0.4</v>
@@ -479,24 +502,24 @@
         <v>25</v>
       </c>
       <c r="E2">
-        <v>3.0461610560024992E-2</v>
+        <v>3.0461610560025001</v>
       </c>
       <c r="F2">
         <v>4.6788399592000012</v>
       </c>
       <c r="M2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" t="s">
         <v>16</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>17</v>
-      </c>
-      <c r="O2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>0.4</v>
@@ -508,13 +531,14 @@
         <v>25</v>
       </c>
       <c r="E3">
-        <v>3.3050847457627118E-2</v>
+        <v>3.3050847457627119</v>
       </c>
       <c r="F3">
         <v>4.6788399592000012</v>
       </c>
       <c r="G3">
-        <v>0.9</v>
+        <f>0.18</f>
+        <v>0.18</v>
       </c>
       <c r="H3">
         <v>0.83299999999999996</v>
@@ -532,18 +556,18 @@
         <v>2.5</v>
       </c>
       <c r="M3" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" t="s">
         <v>20</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>21</v>
-      </c>
-      <c r="O3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4">
         <v>0.56000000000000005</v>
@@ -555,24 +579,24 @@
         <v>25</v>
       </c>
       <c r="E4">
-        <v>3.0687054880603266E-2</v>
+        <v>3.0687054880603264</v>
       </c>
       <c r="F4">
         <v>4.6788399592000012</v>
       </c>
       <c r="M4" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" t="s">
         <v>16</v>
       </c>
-      <c r="N4" t="s">
-        <v>17</v>
-      </c>
       <c r="O4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5">
         <v>0.56000000000000005</v>
@@ -584,13 +608,14 @@
         <v>25</v>
       </c>
       <c r="E5">
-        <v>3.3295454545454538E-2</v>
+        <v>3.3295454545454537</v>
       </c>
       <c r="F5">
         <v>4.6788399592000012</v>
       </c>
       <c r="G5">
-        <v>0.9</v>
+        <f>0.18</f>
+        <v>0.18</v>
       </c>
       <c r="H5">
         <v>0.83299999999999996</v>
@@ -608,18 +633,18 @@
         <v>2.5</v>
       </c>
       <c r="M5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N5" t="s">
         <v>20</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>21</v>
-      </c>
-      <c r="O5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6">
         <v>0.48499999999999999</v>
@@ -631,13 +656,13 @@
         <v>25</v>
       </c>
       <c r="E6">
-        <v>9.2246335944705105E-3</v>
+        <v>0.92246335944705105</v>
       </c>
       <c r="F6">
         <v>3.279208458421452</v>
       </c>
       <c r="G6">
-        <v>0.9</v>
+        <v>0.33300000000000002</v>
       </c>
       <c r="H6">
         <v>0.83299999999999996</v>
@@ -655,58 +680,58 @@
         <v>2.5</v>
       </c>
       <c r="M6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N6" t="s">
+        <v>20</v>
+      </c>
+      <c r="O6" t="s">
         <v>27</v>
-      </c>
-      <c r="N6" t="s">
-        <v>21</v>
-      </c>
-      <c r="O6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7">
         <v>0.43</v>
       </c>
       <c r="E7">
-        <v>9.3528001965583196E-2</v>
+        <v>9.3528001965583201</v>
       </c>
       <c r="F7">
         <v>2.7647690668</v>
       </c>
       <c r="M7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8">
         <v>0.5</v>
       </c>
       <c r="E8">
-        <v>7.230044630753138E-2</v>
+        <v>7.2300446307531381</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9">
         <v>0.12</v>
@@ -715,24 +740,24 @@
         <v>4500000</v>
       </c>
       <c r="E9">
-        <v>2.5595773924911289E-2</v>
+        <v>2.5595773924911289</v>
       </c>
       <c r="F9">
         <v>0</v>
       </c>
       <c r="M9" t="s">
+        <v>33</v>
+      </c>
+      <c r="N9" t="s">
         <v>34</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>35</v>
-      </c>
-      <c r="O9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F10">
         <v>26.573684220000001</v>
@@ -758,45 +783,45 @@
   <sheetData>
     <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="I1" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2">
         <v>0.97</v>
@@ -814,27 +839,27 @@
         <v>20</v>
       </c>
       <c r="G2">
-        <v>3.4299999999999997E-2</v>
-      </c>
-      <c r="H2">
-        <v>9.7699999999999995E-2</v>
+        <v>3.4299999999999997</v>
+      </c>
+      <c r="H2" s="4">
+        <v>9.77</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" t="s">
         <v>42</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>43</v>
-      </c>
-      <c r="L2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3">
         <v>0.61599999999999999</v>
@@ -852,29 +877,29 @@
         <v>20</v>
       </c>
       <c r="G3">
-        <v>1E-4</v>
-      </c>
-      <c r="H3">
-        <v>2.9100000000000001E-2</v>
+        <v>0.01</v>
+      </c>
+      <c r="H3" s="4">
+        <v>2.91</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" t="s">
         <v>46</v>
-      </c>
-      <c r="L3" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Update assumptions for CCGT+CC and SCPC+CC, remove OCGT+CC
</commit_message>
<xml_diff>
--- a/europe/_power/assumptions.xlsx
+++ b/europe/_power/assumptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\31612\MopoProjects\Mopo_WP2_T5_datapipeline_power_20250522\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920418D8-B034-4064-888A-FD0850D17D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DE7501-36D9-4EBC-A8A8-0AA8B1379DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="technology" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
   <si>
     <t>technology</t>
   </si>
@@ -117,9 +117,6 @@
     <t>https://ens.dk/sites/ens.dk/files/Statistik/technology_data_for_el_and_dh_13.xlsx</t>
   </si>
   <si>
-    <t>Base SCPC O&amp;M + efficiency from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
-  </si>
-  <si>
     <t>bioST</t>
   </si>
   <si>
@@ -174,9 +171,6 @@
     <t>https://www.pv-magazine.com/2023/07/14/former-us-coal-plant-to-host-100-hour-iron-air-battery/</t>
   </si>
   <si>
-    <t>Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). | Set eff_in=eff_out=sqrt(RTE) assuming symmetric charge/discharge efficiencies. Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
-  </si>
-  <si>
     <t>investment_cost_energy [EUR/MWh]</t>
   </si>
   <si>
@@ -193,17 +187,45 @@
   </si>
   <si>
     <t>CO2_captured [tCO2/MWh]</t>
+  </si>
+  <si>
+    <t>source_url_3</t>
+  </si>
+  <si>
+    <t>SCPC</t>
+  </si>
+  <si>
+    <t>https://climit.no/app/uploads/sites/4/2019/09/IEAGHG-Report-2019-02-Towards-zero-emissions.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CCS add-on parameters from DEA CCS datasheet '401.a Post comb - small CHP' (amine post-comb capture retrofit). These are generic capture-system assumptions (not gas-specific). CCGT (NGCC) efficiency from IEAGHG report, 48.57% (LHV) with 90% capture rate from Table 20. Investment cost from Table 21.</t>
+  </si>
+  <si>
+    <t>SCPC+CC efficiency from IEAGHG report, net plant (LHV) efficiency with 90% capture rate from Table 17 and costs from Table 18. Base SCPC O&amp;M from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
+  </si>
+  <si>
+    <t>Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -231,6 +253,13 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -249,20 +278,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{2E9EB5C5-2F4E-4BFA-85F0-0B749869C9DB}"/>
   </cellStyles>
@@ -428,20 +463,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="18" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="14.5703125" customWidth="1"/>
     <col min="9" max="9" width="14.140625" customWidth="1"/>
     <col min="10" max="10" width="16.42578125" customWidth="1"/>
     <col min="11" max="11" width="20.140625" customWidth="1"/>
     <col min="12" max="12" width="16.42578125" customWidth="1"/>
-    <col min="13" max="19" width="18" customWidth="1"/>
+    <col min="13" max="20" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -461,7 +499,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>6</v>
@@ -485,26 +523,29 @@
         <v>12</v>
       </c>
       <c r="O1" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="B2">
         <v>0.4</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="6">
         <v>680718.04542770004</v>
       </c>
       <c r="D2">
         <v>25</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="7">
         <v>3.0461610560025001</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="7">
         <v>4.6788399592000012</v>
       </c>
       <c r="M2" t="s">
@@ -513,27 +554,27 @@
       <c r="N2" t="s">
         <v>16</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
       <c r="B3">
         <v>0.4</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="6">
         <v>627389.90362</v>
       </c>
       <c r="D3">
         <v>25</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="7">
         <v>3.3050847457627119</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="7">
         <v>4.6788399592000012</v>
       </c>
       <c r="G3">
@@ -561,27 +602,27 @@
       <c r="N3" t="s">
         <v>20</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>22</v>
       </c>
       <c r="B4">
         <v>0.56000000000000005</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="6">
         <v>1015308.2711464</v>
       </c>
       <c r="D4">
         <v>25</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="7">
         <v>3.0687054880603264</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="7">
         <v>4.6788399592000012</v>
       </c>
       <c r="M4" t="s">
@@ -590,28 +631,28 @@
       <c r="N4" t="s">
         <v>16</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
       <c r="B5">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="C5">
-        <v>935767.99184000015</v>
+        <v>0.48570000000000002</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1704000</v>
       </c>
       <c r="D5">
         <v>25</v>
       </c>
-      <c r="E5">
-        <v>3.3295454545454537</v>
-      </c>
-      <c r="F5">
-        <v>4.6788399592000012</v>
+      <c r="E5" s="7">
+        <v>3.3380281690000002</v>
+      </c>
+      <c r="F5" s="7">
+        <v>12.607127999999999</v>
       </c>
       <c r="G5">
         <f>0.18</f>
@@ -632,34 +673,37 @@
       <c r="L5">
         <v>2.5</v>
       </c>
-      <c r="M5" t="s">
+      <c r="M5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="N5" t="s">
+      <c r="N5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="O5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
       <c r="B6">
-        <v>0.48499999999999999</v>
-      </c>
-      <c r="C6">
-        <v>3800000</v>
+        <v>0.3448</v>
+      </c>
+      <c r="C6" s="6">
+        <v>2808000</v>
       </c>
       <c r="D6">
         <v>25</v>
       </c>
-      <c r="E6">
-        <v>0.92246335944705105</v>
-      </c>
-      <c r="F6">
-        <v>3.279208458421452</v>
+      <c r="E6" s="7">
+        <v>2.7528489999999999</v>
+      </c>
+      <c r="F6" s="7">
+        <v>21.215</v>
       </c>
       <c r="G6">
         <v>0.33300000000000002</v>
@@ -685,85 +729,114 @@
       <c r="N6" t="s">
         <v>20</v>
       </c>
-      <c r="O6" t="s">
+      <c r="O6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>28</v>
       </c>
       <c r="B7">
         <v>0.43</v>
       </c>
-      <c r="E7">
+      <c r="C7" s="6"/>
+      <c r="E7" s="7">
         <v>9.3528001965583201</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="7">
         <v>2.7647690668</v>
       </c>
       <c r="M7" t="s">
         <v>26</v>
       </c>
-      <c r="O7" t="s">
+      <c r="P7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>30</v>
       </c>
       <c r="B8">
         <v>0.5</v>
       </c>
-      <c r="E8">
+      <c r="C8" s="6"/>
+      <c r="E8" s="7">
         <v>7.2300446307531381</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="7">
         <v>0</v>
       </c>
       <c r="M8" t="s">
         <v>26</v>
       </c>
-      <c r="O8" t="s">
+      <c r="P8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>32</v>
       </c>
       <c r="B9">
         <v>0.12</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="6">
         <v>4500000</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="7">
         <v>2.5595773924911289</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="7">
         <v>0</v>
       </c>
       <c r="M9" t="s">
+        <v>32</v>
+      </c>
+      <c r="N9" t="s">
         <v>33</v>
       </c>
-      <c r="N9" t="s">
+      <c r="P9" t="s">
         <v>34</v>
       </c>
-      <c r="O9" t="s">
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>36</v>
-      </c>
-      <c r="F10">
+      <c r="C10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7">
         <v>26.573684220000001</v>
       </c>
     </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11">
+        <v>0.44400000000000001</v>
+      </c>
+      <c r="C11" s="6">
+        <v>1743000</v>
+      </c>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="M5" r:id="rId1" xr:uid="{83F8EEB3-725B-4A44-8915-0382D3CB08F5}"/>
+    <hyperlink ref="N5" r:id="rId2" xr:uid="{251FF512-74F6-4F4B-964D-5D4EAD706837}"/>
+    <hyperlink ref="O5" r:id="rId3" xr:uid="{43E127E0-4748-4E25-B1B4-65B57F71AC2C}"/>
+    <hyperlink ref="O6" r:id="rId4" xr:uid="{A82E2B93-2F7F-4F07-88F4-FB6D3E8EA277}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -771,81 +844,78 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.5703125" customWidth="1"/>
-    <col min="6" max="15" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.5703125" customWidth="1"/>
+    <col min="5" max="14" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>39</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>40</v>
       </c>
       <c r="B2">
         <v>0.97</v>
       </c>
       <c r="C2">
-        <v>0.91</v>
+        <v>245000</v>
       </c>
       <c r="D2">
-        <v>245000</v>
+        <v>86000</v>
       </c>
       <c r="E2">
-        <v>86000</v>
+        <v>20</v>
       </c>
       <c r="F2">
-        <v>20</v>
-      </c>
-      <c r="G2">
         <v>3.4299999999999997</v>
       </c>
-      <c r="H2" s="4">
+      <c r="G2" s="4">
         <v>9.77</v>
       </c>
-      <c r="I2">
+      <c r="H2">
         <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>40</v>
       </c>
       <c r="J2" t="s">
         <v>41</v>
@@ -853,53 +923,47 @@
       <c r="K2" t="s">
         <v>42</v>
       </c>
-      <c r="L2" t="s">
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3">
+        <v>0.63</v>
+      </c>
+      <c r="C3">
+        <v>20000</v>
+      </c>
+      <c r="D3">
+        <v>1900000</v>
+      </c>
+      <c r="E3">
+        <v>20</v>
+      </c>
+      <c r="F3">
+        <v>0.01</v>
+      </c>
+      <c r="G3" s="4">
+        <v>2.91</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" t="s">
         <v>44</v>
       </c>
-      <c r="B3">
-        <v>0.61599999999999999</v>
-      </c>
-      <c r="C3">
-        <v>0.38</v>
-      </c>
-      <c r="D3">
-        <v>20000</v>
-      </c>
-      <c r="E3">
-        <v>550000</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
-      </c>
-      <c r="G3">
-        <v>0.01</v>
-      </c>
-      <c r="H3" s="4">
-        <v>2.91</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
-        <v>51</v>
-      </c>
       <c r="K3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
Add lifetime for existing units to assumptions to account for in decay_capacity
</commit_message>
<xml_diff>
--- a/europe/_power/assumptions.xlsx
+++ b/europe/_power/assumptions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\31612\MopoProjects\Mopo_WP2_T5_datapipeline_power_20250522\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51DE7501-36D9-4EBC-A8A8-0AA8B1379DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6219FC-B023-4071-8BC3-31AE7FAD251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="technology" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="60">
   <si>
     <t>technology</t>
   </si>
@@ -205,6 +205,15 @@
   </si>
   <si>
     <t>Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
+  </si>
+  <si>
+    <t>CCGT</t>
+  </si>
+  <si>
+    <t>nuclear-3</t>
+  </si>
+  <si>
+    <t>oil-eng</t>
   </si>
 </sst>
 </file>
@@ -463,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -744,6 +753,9 @@
         <v>0.43</v>
       </c>
       <c r="C7" s="6"/>
+      <c r="D7">
+        <v>20</v>
+      </c>
       <c r="E7" s="7">
         <v>9.3528001965583201</v>
       </c>
@@ -788,6 +800,9 @@
       <c r="C9" s="6">
         <v>4500000</v>
       </c>
+      <c r="D9">
+        <v>30</v>
+      </c>
       <c r="E9" s="7">
         <v>2.5595773924911289</v>
       </c>
@@ -809,6 +824,9 @@
         <v>35</v>
       </c>
       <c r="C10" s="6"/>
+      <c r="D10">
+        <v>30</v>
+      </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7">
         <v>26.573684220000001</v>
@@ -824,11 +842,34 @@
       <c r="C11" s="6">
         <v>1743000</v>
       </c>
+      <c r="D11">
+        <v>40</v>
+      </c>
       <c r="F11" s="7"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="A12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
change nuclear lifetime assumption to 80 years
</commit_message>
<xml_diff>
--- a/europe/_power/assumptions.xlsx
+++ b/europe/_power/assumptions.xlsx
@@ -1,40 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\31612\MopoProjects\Mopo_WP2_T5_datapipeline_power_20250522\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB6219FC-B023-4071-8BC3-31AE7FAD251D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="technology" sheetId="1" r:id="rId1"/>
-    <sheet name="storage" sheetId="2" r:id="rId2"/>
+    <sheet name="technology" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="storage" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>technology</t>
   </si>
@@ -42,16 +25,19 @@
     <t>conversion_rate</t>
   </si>
   <si>
-    <t>investment_cost [EUR2020/MWh]</t>
+    <t xml:space="preserve">investment_cost [EUR2020/MWh]</t>
   </si>
   <si>
     <t>lifetime</t>
   </si>
   <si>
-    <t>fixed_cost [% investment]</t>
-  </si>
-  <si>
-    <t>operational_cost [EUR2020/MWh]</t>
+    <t xml:space="preserve">fixed_cost [% investment]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operational_cost [EUR2020/MWh]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO2_captured [tCO2/MWh]</t>
   </si>
   <si>
     <t>ccs_heat_MWh_per_tCO2</t>
@@ -75,6 +61,9 @@
     <t>source_url_2</t>
   </si>
   <si>
+    <t>source_url_3</t>
+  </si>
+  <si>
     <t>notes</t>
   </si>
   <si>
@@ -87,7 +76,7 @@
     <t>https://www.sciencedirect.com/science/article/pii/S0360319924023681</t>
   </si>
   <si>
-    <t>H2-fired OCGT: started from DEA natural-gas OCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024) for H2 GT plants. Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
+    <t xml:space="preserve">H2-fired OCGT: started from DEA natural-gas OCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024) for H2 GT plants. Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
   </si>
   <si>
     <t>OCGT+CC</t>
@@ -105,28 +94,37 @@
     <t>CCGT-H2</t>
   </si>
   <si>
-    <t>H2-fired CCGT: started from DEA natural-gas CCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024). Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
+    <t xml:space="preserve">H2-fired CCGT: started from DEA natural-gas CCGT assumptions and applied +8.5% CAPEX uplift from Freitag et al. (2024). Efficiency and O&amp;M left equal to NG as a first-order assumption.</t>
   </si>
   <si>
     <t>CCGT+CC</t>
   </si>
   <si>
+    <t>https://climit.no/app/uploads/sites/4/2019/09/IEAGHG-Report-2019-02-Towards-zero-emissions.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CCS add-on parameters from DEA CCS datasheet '401.a Post comb - small CHP' (amine post-comb capture retrofit). These are generic capture-system assumptions (not gas-specific). CCGT (NGCC) efficiency from IEAGHG report, 48.57% (LHV) with 90% capture rate from Table 20. Investment cost from Table 21.</t>
+  </si>
+  <si>
     <t>SCPC+CC</t>
   </si>
   <si>
     <t>https://ens.dk/sites/ens.dk/files/Statistik/technology_data_for_el_and_dh_13.xlsx</t>
   </si>
   <si>
+    <t xml:space="preserve">SCPC+CC efficiency from IEAGHG report, net plant (LHV) efficiency with 90% capture rate from Table 17 and costs from Table 18. Base SCPC O&amp;M from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
+  </si>
+  <si>
     <t>bioST</t>
   </si>
   <si>
-    <t>Bio steam turbine proxied by DEA 'Biomass CHP - extraction - wood chips - large' (May 2025 Excel).</t>
+    <t xml:space="preserve">Bio steam turbine proxied by DEA 'Biomass CHP - extraction - wood chips - large' (May 2025 Excel).</t>
   </si>
   <si>
     <t>fuelcell</t>
   </si>
   <si>
-    <t>Hydrogen fuel cell proxied by DEA 'Low temp PEM fuel cell - back pressure - hydrogen - small' (May 2025 Excel). Variable O&amp;M = 0 in DEA.</t>
+    <t xml:space="preserve">Hydrogen fuel cell proxied by DEA 'Low temp PEM fuel cell - back pressure - hydrogen - small' (May 2025 Excel). Variable O&amp;M = 0 in DEA.</t>
   </si>
   <si>
     <t>geothermal</t>
@@ -138,19 +136,43 @@
     <t>https://www.irs.gov/individuals/international-taxpayers/yearly-average-currency-exchange-rates</t>
   </si>
   <si>
-    <t>Geothermal fixed O&amp;M from NREL ATB 2024 Geothermal (Hydro/Flash). Converted from 2022 $/kW-yr to EUR/MW-yr using IRS 2022 yearly average (1 USD = 0.951 EUR). Variable O&amp;M assumed 0 (not provided in ATB summary). | Conversion rate set to 12% as representative average across DEA geothermal electricity datasheets (2–5 km depth). DEA reports net electrical efficiencies roughly 10–15% depending on depth; midpoint used. | CAPEX from DEA geothermal electricity datasheets (2–5 km depth). Reported range ≈3–6 M€/MW depending on depth and drilling cost; 4.5 M€/MW used as representative average.</t>
+    <t xml:space="preserve">Geothermal fixed O&amp;M from NREL ATB 2024 Geothermal (Hydro/Flash). Converted from 2022 $/kW-yr to EUR/MW-yr using IRS 2022 yearly average (1 USD = 0.951 EUR). Variable O&amp;M assumed 0 (not provided in ATB summary). | Conversion rate set to 12% as representative average across DEA geothermal electricity datasheets (2–5 km depth). DEA reports net electrical efficiencies roughly 10–15% depending on depth; midpoint used. | CAPEX from DEA geothermal electricity datasheets (2–5 km depth). Reported range ≈3–6 M€/MW depending on depth and drilling cost; 4.5 M€/MW used as representative average.</t>
   </si>
   <si>
     <t>wasteST</t>
   </si>
   <si>
+    <t>SCPC</t>
+  </si>
+  <si>
+    <t>CCGT</t>
+  </si>
+  <si>
+    <t>nuclear-3</t>
+  </si>
+  <si>
+    <t>oil-eng</t>
+  </si>
+  <si>
     <t>storage</t>
   </si>
   <si>
     <t>efficiency</t>
   </si>
   <si>
-    <t>operational_cost [EUR/MWh]</t>
+    <t xml:space="preserve">investment_cost_energy [EUR/MWh]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">investment_cost_power [EUR/MW]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fixed_cost_energy [% investment]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fixed_cost_power [% investment]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">operational_cost [EUR/MWh]</t>
   </si>
   <si>
     <t>battery-storage</t>
@@ -162,112 +184,46 @@
     <t>https://ens.dk/media/6589/download</t>
   </si>
   <si>
-    <t>DEA Energy Storage datasheet '180 Lithium Ion Battery' (Utility-scale). Efficiencies from charge/discharge; capex from 'Specific investment [MEUR2020/MWh]' (2025 ctrl).</t>
+    <t xml:space="preserve">DEA Energy Storage datasheet '180 Lithium Ion Battery' (Utility-scale). Efficiencies from charge/discharge; capex from 'Specific investment [MEUR2020/MWh]' (2025 ctrl).</t>
   </si>
   <si>
     <t>battery-storage-iron-air</t>
   </si>
   <si>
+    <t>https://formenergy.com/technology/</t>
+  </si>
+  <si>
     <t>https://www.pv-magazine.com/2023/07/14/former-us-coal-plant-to-host-100-hour-iron-air-battery/</t>
   </si>
   <si>
-    <t>investment_cost_energy [EUR/MWh]</t>
-  </si>
-  <si>
-    <t>investment_cost_power [EUR/MW]</t>
-  </si>
-  <si>
-    <t>fixed_cost_energy [% investment]</t>
-  </si>
-  <si>
-    <t>fixed_cost_power [% investment]</t>
-  </si>
-  <si>
-    <t>https://formenergy.com/technology/</t>
-  </si>
-  <si>
-    <t>CO2_captured [tCO2/MWh]</t>
-  </si>
-  <si>
-    <t>source_url_3</t>
-  </si>
-  <si>
-    <t>SCPC</t>
-  </si>
-  <si>
-    <t>https://climit.no/app/uploads/sites/4/2019/09/IEAGHG-Report-2019-02-Towards-zero-emissions.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CCS add-on parameters from DEA CCS datasheet '401.a Post comb - small CHP' (amine post-comb capture retrofit). These are generic capture-system assumptions (not gas-specific). CCGT (NGCC) efficiency from IEAGHG report, 48.57% (LHV) with 90% capture rate from Table 20. Investment cost from Table 21.</t>
-  </si>
-  <si>
-    <t>SCPC+CC efficiency from IEAGHG report, net plant (LHV) efficiency with 90% capture rate from Table 17 and costs from Table 18. Base SCPC O&amp;M from DEA el&amp;DH datasheets (May 2025 Excel). CCS-related cost/energy penalty handled via CCS add-on columns. | CAPEX from DEA Electricity &amp; District Heating catalogue + DEA CCS catalogue. SCPC base plant (~2.2–2.5 M€/MW) plus post-combustion capture (~1.3–1.6 M€/MW), total ≈3.5–4.0 M€/MW (4Q2023 EUR).</t>
-  </si>
-  <si>
-    <t>Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
-  </si>
-  <si>
-    <t>CCGT</t>
-  </si>
-  <si>
-    <t>nuclear-3</t>
-  </si>
-  <si>
-    <t>oil-eng</t>
+    <t xml:space="preserve">Iron-air battery (Form Energy) indicative assumptions: 3.5 MW / 350 MWh power block, 100h duration, ~40% AC-AC round-trip efficiency, 20y lifetime from Form Energy presentation; ~$20/kWh is commonly cited as a cost target (not a verified realized project cost). Fixed cost from Form estimate cited by pv-magazine ($19/kW-y), converted using IRS 2023 average 1 USD = 0.924 EUR.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11.000000"/>
+      <color theme="10"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -280,35 +236,34 @@
   </fills>
   <borders count="1">
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+  <cellXfs count="8">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="1" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="2"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{2E9EB5C5-2F4E-4BFA-85F0-0B749869C9DB}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -323,8 +278,291 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -466,135 +704,133 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="16.42578125" customWidth="1"/>
-    <col min="11" max="11" width="20.140625" customWidth="1"/>
-    <col min="12" max="12" width="16.42578125" customWidth="1"/>
-    <col min="13" max="20" width="18" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="19.28515625"/>
+    <col customWidth="1" min="2" max="2" width="17.42578125"/>
+    <col customWidth="1" min="3" max="3" width="18"/>
+    <col customWidth="1" min="4" max="4" width="13"/>
+    <col customWidth="1" min="5" max="7" width="18"/>
+    <col customWidth="1" min="8" max="8" width="14.5703125"/>
+    <col customWidth="1" min="9" max="9" width="14.140625"/>
+    <col customWidth="1" min="10" max="10" width="16.42578125"/>
+    <col customWidth="1" min="11" max="11" width="20.140625"/>
+    <col customWidth="1" min="12" max="12" width="16.42578125"/>
+    <col customWidth="1" min="13" max="20" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="28.5">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="P1" s="3" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B2">
-        <v>0.4</v>
-      </c>
-      <c r="C2" s="6">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="C2" s="2">
         <v>680718.04542770004</v>
       </c>
       <c r="D2">
         <v>25</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="3">
         <v>3.0461610560025001</v>
       </c>
-      <c r="F2" s="7">
+      <c r="F2" s="3">
         <v>4.6788399592000012</v>
       </c>
       <c r="M2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B3">
-        <v>0.4</v>
-      </c>
-      <c r="C3" s="6">
+        <v>0.40000000000000002</v>
+      </c>
+      <c r="C3" s="2">
         <v>627389.90362</v>
       </c>
       <c r="D3">
         <v>25</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="3">
         <v>3.3050847457627119</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="3">
         <v>4.6788399592000012</v>
       </c>
       <c r="G3">
         <f>0.18</f>
-        <v>0.18</v>
+        <v>0.17999999999999999</v>
       </c>
       <c r="H3">
         <v>0.83299999999999996</v>
       </c>
       <c r="I3">
-        <v>0.03</v>
+        <v>0.029999999999999999</v>
       </c>
       <c r="J3">
         <v>8.3000000000000007</v>
@@ -606,72 +842,72 @@
         <v>2.5</v>
       </c>
       <c r="M3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="N3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="P3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4">
         <v>0.56000000000000005</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="2">
         <v>1015308.2711464</v>
       </c>
       <c r="D4">
         <v>25</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="3">
         <v>3.0687054880603264</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="3">
         <v>4.6788399592000012</v>
       </c>
       <c r="M4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B5">
         <v>0.48570000000000002</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="2">
         <v>1704000</v>
       </c>
       <c r="D5">
         <v>25</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="3">
         <v>3.3380281690000002</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="3">
         <v>12.607127999999999</v>
       </c>
       <c r="G5">
         <f>0.18</f>
-        <v>0.18</v>
+        <v>0.17999999999999999</v>
       </c>
       <c r="H5">
         <v>0.83299999999999996</v>
       </c>
       <c r="I5">
-        <v>0.03</v>
+        <v>0.029999999999999999</v>
       </c>
       <c r="J5">
         <v>8.3000000000000007</v>
@@ -682,36 +918,36 @@
       <c r="L5">
         <v>2.5</v>
       </c>
-      <c r="M5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="O5" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="P5" s="8" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B6">
         <v>0.3448</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="2">
         <v>2808000</v>
       </c>
       <c r="D6">
         <v>25</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="3">
         <v>2.7528489999999999</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="3">
         <v>21.215</v>
       </c>
       <c r="G6">
@@ -721,7 +957,7 @@
         <v>0.83299999999999996</v>
       </c>
       <c r="I6">
-        <v>0.03</v>
+        <v>0.029999999999999999</v>
       </c>
       <c r="J6">
         <v>8.3000000000000007</v>
@@ -733,139 +969,139 @@
         <v>2.5</v>
       </c>
       <c r="M6" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="N6" t="s">
-        <v>20</v>
-      </c>
-      <c r="O6" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B7">
-        <v>0.43</v>
-      </c>
-      <c r="C7" s="6"/>
+        <v>0.42999999999999999</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7">
         <v>20</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="3">
         <v>9.3528001965583201</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="3">
         <v>2.7647690668</v>
       </c>
       <c r="M7" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="P7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B8">
         <v>0.5</v>
       </c>
-      <c r="C8" s="6"/>
-      <c r="E8" s="7">
+      <c r="C8" s="2"/>
+      <c r="E8" s="3">
         <v>7.2300446307531381</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="3">
         <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="P8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B9">
         <v>0.12</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="2">
         <v>4500000</v>
       </c>
       <c r="D9">
         <v>30</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="3">
         <v>2.5595773924911289</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="3">
         <v>0</v>
       </c>
       <c r="M9" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="P9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" s="6"/>
+        <v>40</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10">
         <v>30</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7">
+      <c r="E10" s="3"/>
+      <c r="F10" s="3">
         <v>26.573684220000001</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="B11">
         <v>0.44400000000000001</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="2">
         <v>1743000</v>
       </c>
       <c r="D11">
         <v>40</v>
       </c>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="D12">
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="D13">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="D14">
         <v>25</v>
@@ -873,69 +1109,70 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="M5" r:id="rId1" xr:uid="{83F8EEB3-725B-4A44-8915-0382D3CB08F5}"/>
-    <hyperlink ref="N5" r:id="rId2" xr:uid="{251FF512-74F6-4F4B-964D-5D4EAD706837}"/>
-    <hyperlink ref="O5" r:id="rId3" xr:uid="{43E127E0-4748-4E25-B1B4-65B57F71AC2C}"/>
-    <hyperlink ref="O6" r:id="rId4" xr:uid="{A82E2B93-2F7F-4F07-88F4-FB6D3E8EA277}"/>
+    <hyperlink r:id="rId1" ref="M5"/>
+    <hyperlink r:id="rId2" ref="N5"/>
+    <hyperlink r:id="rId3" ref="O5"/>
+    <hyperlink r:id="rId3" ref="O6"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.5703125" customWidth="1"/>
-    <col min="5" max="14" width="18" customWidth="1"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="22.42578125"/>
+    <col customWidth="1" min="2" max="2" width="18"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" width="27.5703125"/>
+    <col customWidth="1" min="4" max="4" width="27.5703125"/>
+    <col customWidth="1" min="5" max="14" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1" ht="30">
+      <c r="A1" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="J1" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K1" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B2">
-        <v>0.97</v>
+        <v>0.96999999999999997</v>
       </c>
       <c r="C2">
         <v>245000</v>
@@ -949,25 +1186,25 @@
       <c r="F2">
         <v>3.4299999999999997</v>
       </c>
-      <c r="G2" s="4">
-        <v>9.77</v>
+      <c r="G2" s="7">
+        <v>9.7699999999999996</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="J2" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B3">
         <v>0.63</v>
@@ -984,28 +1221,29 @@
       <c r="F3">
         <v>0.01</v>
       </c>
-      <c r="G3" s="4">
-        <v>2.91</v>
+      <c r="G3" s="7">
+        <v>2.9100000000000001</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="J3" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="K3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>